<commit_message>
oprava a generovanie a export súboro
Zmeny
Uprava procedúry na generovanie faktúr – doplnenie na 400.
Úprava procedúry na geneovanie výpisov doplnenie čiastočných úhrad 2 splátky z 5 tich.  Pridanie tlačidla na generovanie csv súborov s úhradami do hlavného formulára, oprava logiky dotazu na párovanie splátkových plaltieb. Doplnenie faktúr, znovuvygenerovanie výpisov z banky, znovuexportovanie vybraných tabuliek a dotazov z databázy, uprava dokumentácie.
</commit_message>
<xml_diff>
--- a/export_partneri_aktualizovane.xlsx
+++ b/export_partneri_aktualizovane.xlsx
@@ -442,7 +442,7 @@
       </c>
       <c r="J2" s="0" t="inlineStr">
         <is>
-          <t>SK9509000000000000000006</t>
+          <t>SK9709000000000000000006</t>
         </is>
       </c>
     </row>
@@ -488,11 +488,7 @@
           <t>SK1020524802</t>
         </is>
       </c>
-      <c r="J3" s="0" t="inlineStr">
-        <is>
-          <t>SK8009000000000000000010</t>
-        </is>
-      </c>
+      <c r="J3" s="0" t="inlineStr"/>
     </row>
     <row outlineLevel="0" r="4">
       <c r="A4" s="0">
@@ -536,11 +532,7 @@
           <t>SK2020100587</t>
         </is>
       </c>
-      <c r="J4" s="0" t="inlineStr">
-        <is>
-          <t>SK3309000000000000000011</t>
-        </is>
-      </c>
+      <c r="J4" s="0" t="inlineStr"/>
     </row>
     <row outlineLevel="0" r="5">
       <c r="A5" s="0">
@@ -586,7 +578,7 @@
       </c>
       <c r="J5" s="0" t="inlineStr">
         <is>
-          <t>CZ2601000000000000000019</t>
+          <t>CZ8701000000000000000019</t>
         </is>
       </c>
     </row>
@@ -627,11 +619,7 @@
           <t>GB222777274</t>
         </is>
       </c>
-      <c r="J6" s="0" t="inlineStr">
-        <is>
-          <t>GB46BARC00000000000020</t>
-        </is>
-      </c>
+      <c r="J6" s="0" t="inlineStr"/>
     </row>
     <row outlineLevel="0" r="7">
       <c r="A7" s="0">
@@ -670,11 +658,7 @@
           <t>1087654321</t>
         </is>
       </c>
-      <c r="J7" s="0" t="inlineStr">
-        <is>
-          <t>SK7809000000000000000021</t>
-        </is>
-      </c>
+      <c r="J7" s="0" t="inlineStr"/>
     </row>
     <row outlineLevel="0" r="8">
       <c r="A8" s="0">
@@ -715,7 +699,7 @@
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
-          <t>SK481100000332819938</t>
+          <t>SK2509000000000000000022</t>
         </is>
       </c>
     </row>
@@ -746,6 +730,11 @@
           <t>28055443</t>
         </is>
       </c>
+      <c r="J9" s="0" t="inlineStr">
+        <is>
+          <t>CZ1701000000000000000062</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="10">
       <c r="A10" s="0">
@@ -776,7 +765,7 @@
       </c>
       <c r="J10" s="0" t="inlineStr">
         <is>
-          <t>AT2100000000000000000063</t>
+          <t>AT6900000000000000000063</t>
         </is>
       </c>
     </row>
@@ -809,7 +798,7 @@
       </c>
       <c r="J11" s="0" t="inlineStr">
         <is>
-          <t>DE57100400000000000064</t>
+          <t>DE34100400000000000064</t>
         </is>
       </c>
     </row>
@@ -842,7 +831,7 @@
       </c>
       <c r="J12" s="0" t="inlineStr">
         <is>
-          <t>GB48BARC00000000000065</t>
+          <t>GB46BARC00000000000065</t>
         </is>
       </c>
     </row>
@@ -873,11 +862,7 @@
           <t>44332211</t>
         </is>
       </c>
-      <c r="J13" s="0" t="inlineStr">
-        <is>
-          <t>PL6700000000000000000066</t>
-        </is>
-      </c>
+      <c r="J13" s="0" t="inlineStr"/>
     </row>
     <row outlineLevel="0" r="14">
       <c r="A14" s="0">
@@ -908,7 +893,7 @@
       </c>
       <c r="J14" s="0" t="inlineStr">
         <is>
-          <t>HU1900000000000000000067</t>
+          <t>HU3300000000000000000067</t>
         </is>
       </c>
     </row>
@@ -967,11 +952,7 @@
           <t>77661122</t>
         </is>
       </c>
-      <c r="J16" s="0" t="inlineStr">
-        <is>
-          <t>US37BOFA00000000000069</t>
-        </is>
-      </c>
+      <c r="J16" s="0" t="inlineStr"/>
     </row>
     <row outlineLevel="0" r="17">
       <c r="A17" s="0">
@@ -1028,6 +1009,11 @@
           <t>36554477</t>
         </is>
       </c>
+      <c r="J18" s="0" t="inlineStr">
+        <is>
+          <t>SK6909000000000000000071</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="19">
       <c r="A19" s="0">
@@ -1084,11 +1070,7 @@
           <t>11223399</t>
         </is>
       </c>
-      <c r="J20" s="0" t="inlineStr">
-        <is>
-          <t>SK6509000000000000000073</t>
-        </is>
-      </c>
+      <c r="J20" s="0" t="inlineStr"/>
     </row>
     <row outlineLevel="0" r="21">
       <c r="A21" s="0">
@@ -1173,6 +1155,11 @@
           <t>66778811</t>
         </is>
       </c>
+      <c r="J23" s="0" t="inlineStr">
+        <is>
+          <t>SK8009000000000000000076</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="24">
       <c r="A24" s="0">
@@ -1203,7 +1190,7 @@
       </c>
       <c r="J24" s="0" t="inlineStr">
         <is>
-          <t>SK9909000000000000000077</t>
+          <t>SK4409000000000000000077</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1223,7 @@
       </c>
       <c r="J25" s="0" t="inlineStr">
         <is>
-          <t>SK4409000000000000000078</t>
+          <t>SK4909000000000000000078</t>
         </is>
       </c>
     </row>
@@ -1269,7 +1256,7 @@
       </c>
       <c r="J26" s="0" t="inlineStr">
         <is>
-          <t>SK6209000000000000000079</t>
+          <t>SK9109000000000000000079</t>
         </is>
       </c>
     </row>
@@ -1302,7 +1289,7 @@
       </c>
       <c r="J27" s="0" t="inlineStr">
         <is>
-          <t>SK5609000000000000000080</t>
+          <t>SK8009000000000000000080</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1322,7 @@
       </c>
       <c r="J28" s="0" t="inlineStr">
         <is>
-          <t>IE14BOFI00000000000081</t>
+          <t>IE74BOFI00000000000081</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1355,7 @@
       </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
-          <t>IE72BOFI00000000000082</t>
+          <t>IE91BOFI00000000000082</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1388,7 @@
       </c>
       <c r="J30" s="0" t="inlineStr">
         <is>
-          <t>IE52BOFI00000000000083</t>
+          <t>IE37BOFI00000000000083</t>
         </is>
       </c>
     </row>
@@ -1434,7 +1421,7 @@
       </c>
       <c r="J31" s="0" t="inlineStr">
         <is>
-          <t>GB67BARC00000000000084</t>
+          <t>GB51BARC00000000000084</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1454,7 @@
       </c>
       <c r="J32" s="0" t="inlineStr">
         <is>
-          <t>IE65BOFI00000000000085</t>
+          <t>IE42BOFI00000000000085</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1487,7 @@
       </c>
       <c r="J33" s="0" t="inlineStr">
         <is>
-          <t>GB49BARC00000000000086</t>
+          <t>GB32BARC00000000000086</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1520,7 @@
       </c>
       <c r="J34" s="0" t="inlineStr">
         <is>
-          <t>US20BOFA00000000000087</t>
+          <t>US77BOFA00000000000087</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1553,7 @@
       </c>
       <c r="J35" s="0" t="inlineStr">
         <is>
-          <t>GB42BARC00000000000088</t>
+          <t>GB90BARC00000000000088</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1586,7 @@
       </c>
       <c r="J36" s="0" t="inlineStr">
         <is>
-          <t>SK7209000000000000000089</t>
+          <t>SK9509000000000000000089</t>
         </is>
       </c>
     </row>
@@ -1632,7 +1619,7 @@
       </c>
       <c r="J37" s="0" t="inlineStr">
         <is>
-          <t>SK7509000000000000000090</t>
+          <t>SK1509000000000000000090</t>
         </is>
       </c>
     </row>
@@ -1665,7 +1652,7 @@
       </c>
       <c r="J38" s="0" t="inlineStr">
         <is>
-          <t>SK9609000000000000000091</t>
+          <t>SK8109000000000000000091</t>
         </is>
       </c>
     </row>

</xml_diff>